<commit_message>
feat(nhanvien): Dat mac dinh cot Loai Nhan Vien OFFICER_TYPE la 4
</commit_message>
<xml_diff>
--- a/data/Danh_Muc_Nhan_Vien_Mau.xlsx
+++ b/data/Danh_Muc_Nhan_Vien_Mau.xlsx
@@ -397,100 +397,55 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AE10"/>
+  <dimension ref="A1:P10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>STT</v>
       </c>
       <c r="B1" t="str">
-        <v>MA_NHAN_VIEN</v>
+        <v>OFFICER_NAME</v>
       </c>
       <c r="C1" t="str">
-        <v>OFFICER_NAME</v>
+        <v>DEPT_ID</v>
       </c>
       <c r="D1" t="str">
-        <v>DEPT_ID</v>
+        <v>CHUCDANH</v>
       </c>
       <c r="E1" t="str">
-        <v>CHUCDANH</v>
+        <v>CHUCDANH_NN</v>
       </c>
       <c r="F1" t="str">
-        <v>CHUCDANH_NN</v>
+        <v>OFFICER_TYPE</v>
       </c>
       <c r="G1" t="str">
-        <v>OFFICER_TYPE</v>
+        <v>MA_BAC_SI</v>
       </c>
       <c r="H1" t="str">
-        <v>MA_BAC_SI</v>
+        <v>NGAYCAPCCHN</v>
       </c>
       <c r="I1" t="str">
-        <v>NGAYCAPCCHN</v>
+        <v>NOICAPCCHN</v>
       </c>
       <c r="J1" t="str">
-        <v>NOICAPCCHN</v>
+        <v>CMND</v>
       </c>
       <c r="K1" t="str">
-        <v>CMND</v>
+        <v>SO_BHXH</v>
       </c>
       <c r="L1" t="str">
-        <v>SO_BHXH</v>
+        <v>GIOITINH</v>
       </c>
       <c r="M1" t="str">
-        <v>GIOITINH</v>
+        <v>PHONE</v>
       </c>
       <c r="N1" t="str">
-        <v>PHONE</v>
+        <v>EMAIL</v>
       </c>
       <c r="O1" t="str">
-        <v>EMAIL</v>
+        <v>TGLAMVIECTUAN</v>
       </c>
       <c r="P1" t="str">
-        <v>MA_KHOA</v>
-      </c>
-      <c r="Q1" t="str">
-        <v>VITRICHUYENMON</v>
-      </c>
-      <c r="R1" t="str">
-        <v>PHAMVI_CHUYENMON</v>
-      </c>
-      <c r="S1" t="str">
-        <v>SOQDPHAMVIHANHNGHE</v>
-      </c>
-      <c r="T1" t="str">
-        <v>DVKTPHANCONGTH</v>
-      </c>
-      <c r="U1" t="str">
-        <v>SOQDDVKTPHANCONGTH</v>
-      </c>
-      <c r="V1" t="str">
-        <v>TGDANGKYHANHNGHE</v>
-      </c>
-      <c r="W1" t="str">
-        <v>TGLAMVIECNGAY</v>
-      </c>
-      <c r="X1" t="str">
-        <v>TGLAMVIECTUAN</v>
-      </c>
-      <c r="Y1" t="str">
-        <v>CSLAMVIECKHAC</v>
-      </c>
-      <c r="Z1" t="str">
-        <v>QDCHUYENGIAOKT</v>
-      </c>
-      <c r="AA1" t="str">
-        <v>TUNGAY</v>
-      </c>
-      <c r="AB1" t="str">
-        <v>DENNGAY</v>
-      </c>
-      <c r="AC1" t="str">
-        <v>DMGUIBH</v>
-      </c>
-      <c r="AD1" t="str">
-        <v>NGAYCHECKGUIBH</v>
-      </c>
-      <c r="AE1" t="str">
         <v>STATUS</v>
       </c>
     </row>
@@ -498,49 +453,49 @@
       <c r="A2">
         <v>1</v>
       </c>
+      <c r="B2" t="str">
+        <v>Quàng Thị Dung</v>
+      </c>
       <c r="C2" t="str">
-        <v>Quàng Thị Dung</v>
+        <v>Điểm TYT xã Mường Pồn</v>
       </c>
       <c r="D2" t="str">
-        <v>Điểm TYT xã Mường Pồn</v>
-      </c>
-      <c r="E2" t="str">
         <v>Y sỹ đa khoa</v>
       </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
       <c r="F2">
-        <v>2</v>
-      </c>
-      <c r="G2">
-        <v>14</v>
-      </c>
-      <c r="H2" t="str">
+        <v>4</v>
+      </c>
+      <c r="G2" t="str">
         <v>0002205/ĐB-CCHN</v>
       </c>
-      <c r="I2">
+      <c r="H2">
         <v>44072.29201388889</v>
       </c>
-      <c r="J2" t="str">
+      <c r="I2" t="str">
         <v>SYT tỉnh Điện Biên</v>
+      </c>
+      <c r="J2">
+        <v>11185003116</v>
       </c>
       <c r="K2">
         <v>11185003116</v>
       </c>
       <c r="L2">
-        <v>11185003116</v>
+        <v>2</v>
       </c>
       <c r="M2">
-        <v>2</v>
-      </c>
-      <c r="N2">
         <v>931654118</v>
       </c>
+      <c r="N2" t="str">
+        <v>quangdung031985@gmail.com</v>
+      </c>
       <c r="O2" t="str">
-        <v>quangdung031985@gmail.com</v>
-      </c>
-      <c r="X2" t="str">
         <v>T2T3T4T5T6</v>
       </c>
-      <c r="AE2">
+      <c r="P2">
         <v>1</v>
       </c>
     </row>
@@ -548,49 +503,49 @@
       <c r="A3">
         <v>2</v>
       </c>
+      <c r="B3" t="str">
+        <v>Nguyễn Thị Nhung</v>
+      </c>
       <c r="C3" t="str">
-        <v>Nguyễn Thị Nhung</v>
+        <v>Điểm TYT xã Mường Pồn</v>
       </c>
       <c r="D3" t="str">
-        <v>Điểm TYT xã Mường Pồn</v>
-      </c>
-      <c r="E3" t="str">
         <v>CNYTCC</v>
       </c>
+      <c r="E3">
+        <v>4</v>
+      </c>
       <c r="F3">
         <v>4</v>
       </c>
-      <c r="G3">
-        <v>14</v>
-      </c>
-      <c r="H3" t="str">
+      <c r="G3" t="str">
         <v>0001067/ĐB-CCHN</v>
       </c>
-      <c r="I3">
+      <c r="H3">
         <v>44071.29201388889</v>
       </c>
-      <c r="J3" t="str">
+      <c r="I3" t="str">
         <v>SYT tỉnh Điện Biên</v>
+      </c>
+      <c r="J3">
+        <v>1187039166</v>
       </c>
       <c r="K3">
         <v>1187039166</v>
       </c>
       <c r="L3">
-        <v>1187039166</v>
+        <v>2</v>
       </c>
       <c r="M3">
-        <v>2</v>
-      </c>
-      <c r="N3">
         <v>339106288</v>
       </c>
+      <c r="N3" t="str">
+        <v>nguyennhungytdb@gmail.com.</v>
+      </c>
       <c r="O3" t="str">
-        <v>nguyennhungytdb@gmail.com.</v>
-      </c>
-      <c r="X3" t="str">
         <v>T2T3T4T5T6</v>
       </c>
-      <c r="AE3">
+      <c r="P3">
         <v>1</v>
       </c>
     </row>
@@ -598,49 +553,49 @@
       <c r="A4">
         <v>3</v>
       </c>
+      <c r="B4" t="str">
+        <v>Lò Thị Liên</v>
+      </c>
       <c r="C4" t="str">
-        <v>Lò Thị Liên</v>
+        <v>Điểm TYT xã Mường Pồn</v>
       </c>
       <c r="D4" t="str">
-        <v>Điểm TYT xã Mường Pồn</v>
-      </c>
-      <c r="E4" t="str">
         <v>Hộ sinh cao đẳng</v>
       </c>
+      <c r="E4">
+        <v>4</v>
+      </c>
       <c r="F4">
         <v>4</v>
       </c>
-      <c r="G4">
-        <v>14</v>
-      </c>
-      <c r="H4" t="str">
+      <c r="G4" t="str">
         <v>002510/ĐB-CCHN</v>
       </c>
-      <c r="I4">
+      <c r="H4">
         <v>44747.29201388889</v>
       </c>
-      <c r="J4" t="str">
+      <c r="I4" t="str">
         <v>SYT tỉnh Điện Biên</v>
+      </c>
+      <c r="J4">
+        <v>11184003522</v>
       </c>
       <c r="K4">
         <v>11184003522</v>
       </c>
       <c r="L4">
-        <v>11184003522</v>
+        <v>2</v>
       </c>
       <c r="M4">
-        <v>2</v>
-      </c>
-      <c r="N4">
         <v>353103343</v>
       </c>
+      <c r="N4" t="str">
+        <v>liendb6688@gmal.com</v>
+      </c>
       <c r="O4" t="str">
-        <v>liendb6688@gmal.com</v>
-      </c>
-      <c r="X4" t="str">
         <v>T2T3T4T5T6</v>
       </c>
-      <c r="AE4">
+      <c r="P4">
         <v>1</v>
       </c>
     </row>
@@ -648,49 +603,49 @@
       <c r="A5">
         <v>4</v>
       </c>
+      <c r="B5" t="str">
+        <v>Nguyễn Đức Thoại</v>
+      </c>
       <c r="C5" t="str">
-        <v>Nguyễn Đức Thoại</v>
+        <v>Điểm TYT xã Mường Pồn</v>
       </c>
       <c r="D5" t="str">
-        <v>Điểm TYT xã Mường Pồn</v>
-      </c>
-      <c r="E5" t="str">
         <v>Dược sỹ cao đẳng</v>
       </c>
+      <c r="E5">
+        <v>8</v>
+      </c>
       <c r="F5">
-        <v>8</v>
-      </c>
-      <c r="G5">
-        <v>8</v>
-      </c>
-      <c r="H5" t="str">
+        <v>4</v>
+      </c>
+      <c r="G5" t="str">
         <v>561/ĐB-CCHN</v>
       </c>
-      <c r="I5">
+      <c r="H5">
         <v>44746.29201388889</v>
       </c>
-      <c r="J5" t="str">
+      <c r="I5" t="str">
         <v>SYT tỉnh Điện Biên</v>
+      </c>
+      <c r="J5">
+        <v>11091004880</v>
       </c>
       <c r="K5">
         <v>11091004880</v>
       </c>
       <c r="L5">
-        <v>11091004880</v>
+        <v>1</v>
       </c>
       <c r="M5">
-        <v>1</v>
-      </c>
-      <c r="N5">
         <v>914445151</v>
       </c>
+      <c r="N5" t="str">
+        <v>thoaid3a.tt@gmail.com</v>
+      </c>
       <c r="O5" t="str">
-        <v>thoaid3a.tt@gmail.com</v>
-      </c>
-      <c r="X5" t="str">
         <v>T2T3T4T5T6</v>
       </c>
-      <c r="AE5">
+      <c r="P5">
         <v>1</v>
       </c>
     </row>
@@ -698,49 +653,49 @@
       <c r="A6">
         <v>5</v>
       </c>
+      <c r="B6" t="str">
+        <v>Lò Văn Bích</v>
+      </c>
       <c r="C6" t="str">
-        <v>Lò Văn Bích</v>
+        <v>Điểm TYT xã Mường Pồn</v>
       </c>
       <c r="D6" t="str">
-        <v>Điểm TYT xã Mường Pồn</v>
-      </c>
-      <c r="E6" t="str">
         <v>Y sỹ đa khoa</v>
       </c>
+      <c r="E6">
+        <v>2</v>
+      </c>
       <c r="F6">
-        <v>2</v>
-      </c>
-      <c r="G6">
-        <v>14</v>
-      </c>
-      <c r="H6" t="str">
+        <v>4</v>
+      </c>
+      <c r="G6" t="str">
         <v>002980/ĐB-CCHN</v>
       </c>
-      <c r="I6">
+      <c r="H6">
         <v>43798.29201388889</v>
       </c>
-      <c r="J6" t="str">
+      <c r="I6" t="str">
         <v>SYT tỉnh Điện Biên</v>
+      </c>
+      <c r="J6">
+        <v>11066000219</v>
       </c>
       <c r="K6">
         <v>11066000219</v>
       </c>
       <c r="L6">
-        <v>11066000219</v>
+        <v>1</v>
       </c>
       <c r="M6">
-        <v>1</v>
-      </c>
-      <c r="N6">
         <v>358047611</v>
       </c>
+      <c r="N6" t="str">
+        <v>lobich1966@gmail.com</v>
+      </c>
       <c r="O6" t="str">
-        <v>lobich1966@gmail.com</v>
-      </c>
-      <c r="X6" t="str">
         <v>T2T3T4T5T6</v>
       </c>
-      <c r="AE6">
+      <c r="P6">
         <v>1</v>
       </c>
     </row>
@@ -748,49 +703,49 @@
       <c r="A7">
         <v>6</v>
       </c>
+      <c r="B7" t="str">
+        <v>Quàng Thị Chung</v>
+      </c>
       <c r="C7" t="str">
-        <v>Quàng Thị Chung</v>
+        <v>Điểm TYT xã Mường Pồn</v>
       </c>
       <c r="D7" t="str">
-        <v>Điểm TYT xã Mường Pồn</v>
-      </c>
-      <c r="E7" t="str">
         <v>Cử nhân dân số</v>
       </c>
+      <c r="E7">
+        <v>2</v>
+      </c>
       <c r="F7">
-        <v>2</v>
-      </c>
-      <c r="G7">
-        <v>14</v>
-      </c>
-      <c r="H7" t="str">
+        <v>4</v>
+      </c>
+      <c r="G7" t="str">
         <v>0002204/ĐB-CCHN</v>
       </c>
-      <c r="I7">
+      <c r="H7">
         <v>44072.29201388889</v>
       </c>
-      <c r="J7" t="str">
+      <c r="I7" t="str">
         <v>SYT tỉnh Điện Biên</v>
+      </c>
+      <c r="J7">
+        <v>11189002952</v>
       </c>
       <c r="K7">
         <v>11189002952</v>
       </c>
       <c r="L7">
-        <v>11189002952</v>
+        <v>2</v>
       </c>
       <c r="M7">
-        <v>2</v>
-      </c>
-      <c r="N7">
         <v>919331089</v>
       </c>
+      <c r="N7" t="str">
+        <v>quangthichung1989@gmail.com</v>
+      </c>
       <c r="O7" t="str">
-        <v>quangthichung1989@gmail.com</v>
-      </c>
-      <c r="X7" t="str">
         <v>T2T3T4T5T6</v>
       </c>
-      <c r="AE7">
+      <c r="P7">
         <v>1</v>
       </c>
     </row>
@@ -798,37 +753,37 @@
       <c r="A8">
         <v>7</v>
       </c>
+      <c r="B8" t="str">
+        <v>Lò Thị Phiến</v>
+      </c>
       <c r="C8" t="str">
-        <v>Lò Thị Phiến</v>
+        <v>Điểm TYT xã Mường Pồn</v>
       </c>
       <c r="D8" t="str">
-        <v>Điểm TYT xã Mường Pồn</v>
-      </c>
-      <c r="E8" t="str">
         <v>Cử nhân dân số</v>
       </c>
-      <c r="G8">
-        <v>14</v>
+      <c r="F8">
+        <v>4</v>
+      </c>
+      <c r="J8">
+        <v>11189000665</v>
       </c>
       <c r="K8">
         <v>11189000665</v>
       </c>
       <c r="L8">
-        <v>11189000665</v>
+        <v>2</v>
       </c>
       <c r="M8">
-        <v>2</v>
-      </c>
-      <c r="N8">
         <v>353466933</v>
       </c>
+      <c r="N8" t="str">
+        <v>lophiends@gmail.com.</v>
+      </c>
       <c r="O8" t="str">
-        <v>lophiends@gmail.com.</v>
-      </c>
-      <c r="X8" t="str">
         <v>T2T3T4T5T6</v>
       </c>
-      <c r="AE8">
+      <c r="P8">
         <v>1</v>
       </c>
     </row>
@@ -836,37 +791,37 @@
       <c r="A9">
         <v>8</v>
       </c>
+      <c r="B9" t="str">
+        <v>Mùa A Páo</v>
+      </c>
       <c r="C9" t="str">
-        <v>Mùa A Páo</v>
+        <v>Điểm TYT xã Mường Pồn</v>
       </c>
       <c r="D9" t="str">
-        <v>Điểm TYT xã Mường Pồn</v>
-      </c>
-      <c r="E9" t="str">
         <v>Cử nhân dinh dưỡng</v>
       </c>
-      <c r="G9">
-        <v>14</v>
+      <c r="F9">
+        <v>4</v>
+      </c>
+      <c r="J9">
+        <v>11086000428</v>
       </c>
       <c r="K9">
         <v>11086000428</v>
       </c>
       <c r="L9">
-        <v>11086000428</v>
+        <v>1</v>
       </c>
       <c r="M9">
-        <v>1</v>
-      </c>
-      <c r="N9">
         <v>384053322</v>
       </c>
+      <c r="N9" t="str">
+        <v>paotytmuongpon@gmail.com.</v>
+      </c>
       <c r="O9" t="str">
-        <v>paotytmuongpon@gmail.com.</v>
-      </c>
-      <c r="X9" t="str">
         <v>T2T3T4T5T6</v>
       </c>
-      <c r="AE9">
+      <c r="P9">
         <v>1</v>
       </c>
     </row>
@@ -874,55 +829,55 @@
       <c r="A10">
         <v>9</v>
       </c>
+      <c r="B10" t="str">
+        <v>Tòng Thị Thơ</v>
+      </c>
       <c r="C10" t="str">
-        <v>Tòng Thị Thơ</v>
+        <v>Điểm TYT xã Mường Pồn</v>
       </c>
       <c r="D10" t="str">
-        <v>Điểm TYT xã Mường Pồn</v>
-      </c>
-      <c r="E10" t="str">
         <v>Điều dưỡng cao đẳng</v>
       </c>
+      <c r="E10">
+        <v>3</v>
+      </c>
       <c r="F10">
-        <v>3</v>
-      </c>
-      <c r="G10">
-        <v>6</v>
-      </c>
-      <c r="H10" t="str">
+        <v>4</v>
+      </c>
+      <c r="G10" t="str">
         <v>000022/ĐB-CCHN</v>
       </c>
-      <c r="I10">
+      <c r="H10">
         <v>44859.29201388889</v>
       </c>
-      <c r="J10" t="str">
+      <c r="I10" t="str">
         <v>SYT tỉnh Điện Biên</v>
+      </c>
+      <c r="J10">
+        <v>11189004835</v>
       </c>
       <c r="K10">
         <v>11189004835</v>
       </c>
       <c r="L10">
-        <v>11189004835</v>
+        <v>2</v>
       </c>
       <c r="M10">
-        <v>2</v>
-      </c>
-      <c r="N10">
         <v>346458988</v>
       </c>
+      <c r="N10" t="str">
+        <v>thotong1989@gmail.com</v>
+      </c>
       <c r="O10" t="str">
-        <v>thotong1989@gmail.com</v>
-      </c>
-      <c r="X10" t="str">
         <v>T2T3T4T5T6</v>
       </c>
-      <c r="AE10">
+      <c r="P10">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AE10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>